<commit_message>
Added controller for Mobiliser view
</commit_message>
<xml_diff>
--- a/SourceFiles/UserDetails.xlsx
+++ b/SourceFiles/UserDetails.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GGupta\Desktop\GFEDTechTitans-Git\SourceFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PGaur\source\repos\GFEDTechTitans\SourceFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED3F7DD0-DDA1-4675-A9D2-F0267A2B1E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759F0CB8-684B-4ACB-B744-01109985410B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="705" yWindow="705" windowWidth="34560" windowHeight="13545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57120" windowHeight="21180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDetails" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>UserId</t>
   </si>
@@ -43,6 +43,12 @@
   </si>
   <si>
     <t>Gopesh Gupta</t>
+  </si>
+  <si>
+    <t>Preeti Gaur</t>
+  </si>
+  <si>
+    <t>Pgaur</t>
   </si>
 </sst>
 </file>
@@ -360,7 +366,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
@@ -391,6 +397,14 @@
         <v>5</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>